<commit_message>
Create performance model for reduction operators (#545)
Fixes #533

The performance model is currently bare-bones, based on O(n) operations
being strictly necessary for these reductions.

It could be more tuned but that would depend significantly on the
implementation and the theoretical limit is something like n/2 + log(n)
at a minimum which is not likely significantly more accurate

---------

Co-authored-by: Copilot Autofix powered by AI <175728472+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/traces/h100/facebook_timesformer-base-finetuned-k400__1016002_perf_report.xlsx
+++ b/tests/traces/h100/facebook_timesformer-base-finetuned-k400__1016002_perf_report.xlsx
@@ -1,22 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gpu_timeline" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ops_summary_by_category" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ops_summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ops_unique_args" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="unified_perf_summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GEMM" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONV_fwd" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BinaryElementwise" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UnaryElementwise" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalization" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="gpu_timeline" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ops_summary_by_category" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ops_summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ops_unique_args" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="unified_perf_summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="GEMM" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CONV_fwd" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="BinaryElementwise" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="UnaryElementwise" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Normalization" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Reduce_fwd" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="kernel_summary" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="short_kernel_histogram" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="short_kernels_summary" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1739,6 +1743,2739 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AJ2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>param: num_input_elems</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>param: num_output_elems</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>param: dtype_in_out</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>param: reduce_type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>GFLOPS_first</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Data Moved (MB)_first</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>FLOPS/Byte_first</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>TB/s_mean</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>TB/s_median</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>TB/s_std</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>TB/s_min</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>TB/s_max</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>TFLOPS/s_mean</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>TFLOPS/s_median</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>TFLOPS/s_std</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>TFLOPS/s_min</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>TFLOPS/s_max</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>process_name_first</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>process_label_first</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>thread_name_first</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Compute Spec</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>kernel_details__summarize_kernel_stats</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>trunc_kernel_details</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Input Dims_first</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Input type_first</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Input Strides_first</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Concrete Inputs_first</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel Time (µs)_mean</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel Time (µs)_median</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel Time (µs)_std</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel Time (µs)_min</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel Time (µs)_max</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel Time (µs)_sum</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>name_count</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>UID_first</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>aten::mean</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>6144</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>('c10::BFloat16', None)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>6.144e-06</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.01172065734863281</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.4999186330349878</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.00226974951117672</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.002259215510277354</v>
+      </c>
+      <c r="K2" t="n">
+        <v>3.751008785294355e-05</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.002220059095920617</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.002341823595087458</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.001134690072959298</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.001129423929629297</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1.875199184446587e-05</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.001109848908489526</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.001170721250465203</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>python3</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>thread 17751 (python3)</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>vector_bf16</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>[{'name': 'void at::native::reduce_kernel&lt;128, 4, at::native::ReduceOp&lt;c10::BFloat16, at::native::MeanOps&lt;c10::BFloat16, float, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt; &gt;(at::native::ReduceOp&lt;c10::BFloat16, at::native::MeanOps&lt;c10::BFloat16, float, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt;)', 'stream': 7, 'count': 12, 'total_duration_us': np.float64(64.99300000000001), 'mean_duration_us': np.float64(5.416083333333334), 'median_duration_us': np.float64(5.44), 'std_dev_duration_us': np.float64(0.08484540680293502), 'min_duration_us': np.float64(5.248), 'max_duration_us': np.float64(5.536)}]</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>[{'name': 'void at::native::reduce_kernel&lt;128, 4, at::native::ReduceOp&lt;c10:...', 'stream': 7, 'mean_duration_us': np.float64(5.42)}]</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>[[1, 8, 768], [], [], []]</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>['c10::BFloat16', 'ScalarList', 'Scalar', '']</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>[[19273728, 2409216, 1], [], [], []]</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>['', '[1]', 'True', '']</t>
+        </is>
+      </c>
+      <c r="AC2" t="n">
+        <v>5.416035970052083</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>5.43994140625</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0.08856812165190991</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>5.248046875</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>5.535888671875</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>64.992431640625</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>12</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>305</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parent op category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Parent cpu_op</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel stream</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel duration (µs)_sum</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel duration (µs)_count</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel duration (µs)_mean</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel duration (µs)_min</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel duration (µs)_max</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Percent of kernels time (%)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Percent of total time (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>aten::_softmax</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>void at::native::(anonymous namespace)::cunn_SoftMaxForward&lt;8, c10::BFloat16, float, c10::BFloat16, at::native::(anonymous namespace)::SoftMaxForwardEpilogue&gt;(c10::BFloat16*, c10::BFloat16 const*, int)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" t="n">
+        <v>68688.625</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5724.052083333333</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5701.537</v>
+      </c>
+      <c r="I2" t="n">
+        <v>5767.809</v>
+      </c>
+      <c r="J2" t="n">
+        <v>44.35656651605</v>
+      </c>
+      <c r="K2" t="n">
+        <v>42.93242273521919</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GEMM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>aten::bmm</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>void cutlass::Kernel2&lt;cutlass_75_tensorop_bf16_s1688gemm_bf16_128x128_nn_align1&gt;(cutlass_75_tensorop_bf16_s1688gemm_bf16_128x128_nn_align1::Params)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3" t="n">
+        <v>43207.642</v>
+      </c>
+      <c r="F3" t="n">
+        <v>24</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1800.318416666667</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1682.295</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1919.478</v>
+      </c>
+      <c r="J3" t="n">
+        <v>27.90189272786689</v>
+      </c>
+      <c r="K3" t="n">
+        <v>27.00605452119636</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>elementwise</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>aten::mul</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::native::AUnaryFunctor&lt;c10::BFloat16, c10::BFloat16, c10::BFloat16, at::native::binary_internal::MulFunctor&lt;float&gt; &gt;, std::array&lt;char*, 2ul&gt; &gt;(int, at::native::AUnaryFunctor&lt;c10::BFloat16, c10::BFloat16, c10::BFloat16, at::native::binary_internal::MulFunctor&lt;float&gt; &gt;, std::array&lt;char*, 2ul&gt;)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" t="n">
+        <v>15555.788</v>
+      </c>
+      <c r="F4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G4" t="n">
+        <v>648.1578333333333</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4.896</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1292.505</v>
+      </c>
+      <c r="J4" t="n">
+        <v>10.0453509606805</v>
+      </c>
+      <c r="K4" t="n">
+        <v>9.72282770830614</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GEMM</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>aten::addmm</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>sm90_xmma_gemm_bf16bf16_bf16f32_f32_tn_n_tilesize128x128x64_warpgroupsize1x1x1_execute_segment_k_off_kernel__5x_cublas</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" t="n">
+        <v>8486.164000000001</v>
+      </c>
+      <c r="F5" t="n">
+        <v>84</v>
+      </c>
+      <c r="G5" t="n">
+        <v>101.0257619047619</v>
+      </c>
+      <c r="H5" t="n">
+        <v>44.992</v>
+      </c>
+      <c r="I5" t="n">
+        <v>165.887</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5.480049978174828</v>
+      </c>
+      <c r="K5" t="n">
+        <v>5.304103557880197</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>elementwise</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>aten::copy_</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1}&gt;(at::TensorIteratorBase&amp;, at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1} const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1}&gt;(at::TensorIteratorBase&amp;, at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1} const&amp;)::{lambda(int)#1})</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>7378.101</v>
+      </c>
+      <c r="F6" t="n">
+        <v>122</v>
+      </c>
+      <c r="G6" t="n">
+        <v>60.47623770491803</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2.944</v>
+      </c>
+      <c r="I6" t="n">
+        <v>154.079</v>
+      </c>
+      <c r="J6" t="n">
+        <v>4.764503988377043</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4.611531401525994</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NORM_fwd</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>aten::native_layer_norm</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>void at::native::(anonymous namespace)::vectorized_layer_norm_kernel&lt;c10::BFloat16, float&gt;(int, float, c10::BFloat16 const*, c10::BFloat16 const*, c10::BFloat16 const*, float*, float*, c10::BFloat16*)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2202.649</v>
+      </c>
+      <c r="F7" t="n">
+        <v>37</v>
+      </c>
+      <c r="G7" t="n">
+        <v>59.53105405405405</v>
+      </c>
+      <c r="H7" t="n">
+        <v>58.815</v>
+      </c>
+      <c r="I7" t="n">
+        <v>60.544</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1.422389032827648</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1.376720788999748</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>aten::cat</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>void at::native::(anonymous namespace)::CatArrayBatchedCopy_contig&lt;at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;, unsigned int, 3, 128, 1&gt;(at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;*, at::native::(anonymous namespace)::CatArrInputTensorMetadata&lt;at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;, unsigned int, 128, 1&gt;, at::native::(anonymous namespace)::TensorSizeStride&lt;unsigned int, 4u&gt;, int, unsigned int)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1780.948</v>
+      </c>
+      <c r="F8" t="n">
+        <v>25</v>
+      </c>
+      <c r="G8" t="n">
+        <v>71.23791999999999</v>
+      </c>
+      <c r="H8" t="n">
+        <v>69.983</v>
+      </c>
+      <c r="I8" t="n">
+        <v>72.223</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.150070166983634</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.113145188238127</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>elementwise</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>aten::gelu</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::native::GeluCUDAKernelImpl(at::TensorIteratorBase&amp;, at::native::GeluType)::{lambda()#2}::operator()() const::{lambda()#4}::operator()() const::{lambda(c10::BFloat16)#1}, std::array&lt;char*, 2ul&gt; &gt;(int, at::native::GeluCUDAKernelImpl(at::TensorIteratorBase&amp;, at::native::GeluType)::{lambda()#2}::operator()() const::{lambda()#4}::operator()() const::{lambda(c10::BFloat16)#1}, std::array&lt;char*, 2ul&gt;)</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1534.2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" t="n">
+        <v>127.85</v>
+      </c>
+      <c r="H9" t="n">
+        <v>127.103</v>
+      </c>
+      <c r="I9" t="n">
+        <v>128.703</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.9907294599203859</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.9589203883521221</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>elementwise</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>aten::add</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt;, std::array&lt;char*, 3ul&gt; &gt;(int, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt;, std::array&lt;char*, 3ul&gt;)</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1360.379</v>
+      </c>
+      <c r="F10" t="n">
+        <v>36</v>
+      </c>
+      <c r="G10" t="n">
+        <v>37.78830555555556</v>
+      </c>
+      <c r="H10" t="n">
+        <v>35.04</v>
+      </c>
+      <c r="I10" t="n">
+        <v>39.936</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.8784823047562473</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.8502771209660224</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>aten::cat</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>void at::native::(anonymous namespace)::CatArrayBatchedCopy&lt;at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;, unsigned int, 3, 64, 64&gt;(at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;*, at::native::(anonymous namespace)::CatArrInputTensorMetadata&lt;at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;, unsigned int, 64, 64&gt;, at::native::(anonymous namespace)::TensorSizeStride&lt;unsigned int, 4u&gt;, int, unsigned int)</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1302.169</v>
+      </c>
+      <c r="F11" t="n">
+        <v>13</v>
+      </c>
+      <c r="G11" t="n">
+        <v>100.1668461538462</v>
+      </c>
+      <c r="H11" t="n">
+        <v>93.82299999999999</v>
+      </c>
+      <c r="I11" t="n">
+        <v>161.311</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.8408924456362071</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.8138941488594019</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GEMM</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>aten::bmm</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>void cutlass::Kernel2&lt;cutlass_80_wmma_tensorop_bf16_s161616gemm_bf16_16x16_32x1_nn_align8&gt;(cutlass_80_wmma_tensorop_bf16_s161616gemm_bf16_16x16_32x1_nn_align8::Params)</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>7</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1300.504</v>
+      </c>
+      <c r="F12" t="n">
+        <v>12</v>
+      </c>
+      <c r="G12" t="n">
+        <v>108.3753333333333</v>
+      </c>
+      <c r="H12" t="n">
+        <v>107.583</v>
+      </c>
+      <c r="I12" t="n">
+        <v>109.599</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.8398172503873689</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.812853474601413</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CONV_fwd</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>aten::cudnn_convolution</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>void cutlass__5x_cudnn::Kernel&lt;cutlass_tensorop_bf16_s16816fprop_optimized_bf16_256x64_32x4_nhwc_align8&gt;(cutlass_tensorop_bf16_s16816fprop_optimized_bf16_256x64_32x4_nhwc_align8::Params)</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>7</v>
+      </c>
+      <c r="E13" t="n">
+        <v>863.099</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>863.099</v>
+      </c>
+      <c r="H13" t="n">
+        <v>863.099</v>
+      </c>
+      <c r="I13" t="n">
+        <v>863.099</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.557357323769929</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.5394624092467268</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GEMM</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>aten::bmm</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>void cutlass::Kernel2&lt;cutlass_80_wmma_tensorop_bf16_s161616gemm_bf16_16x16_64x1_nn_align8&gt;(cutlass_80_wmma_tensorop_bf16_s161616gemm_bf16_16x16_64x1_nn_align8::Params)</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E14" t="n">
+        <v>490.207</v>
+      </c>
+      <c r="F14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G14" t="n">
+        <v>40.85058333333333</v>
+      </c>
+      <c r="H14" t="n">
+        <v>40.288</v>
+      </c>
+      <c r="I14" t="n">
+        <v>41.632</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.3165574999082209</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.3063938774689928</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CONV_fwd</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>aten::cudnn_convolution</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>void cudnn::engines_precompiled::nchwToNhwcKernel&lt;__nv_bfloat16, __nv_bfloat16, float, false, true, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nchw2nhwc_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E15" t="n">
+        <v>291.679</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" t="n">
+        <v>145.8395</v>
+      </c>
+      <c r="H15" t="n">
+        <v>10.336</v>
+      </c>
+      <c r="I15" t="n">
+        <v>281.343</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.1883554804719842</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.1823080041416756</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>elementwise</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>aten::add</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>7</v>
+      </c>
+      <c r="E16" t="n">
+        <v>140.063</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" t="n">
+        <v>70.03149999999999</v>
+      </c>
+      <c r="H16" t="n">
+        <v>53.983</v>
+      </c>
+      <c r="I16" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.09044749077358166</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.08754351867668052</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>aten::_softmax</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>void (anonymous namespace)::softmax_warp_forward&lt;c10::BFloat16, c10::BFloat16, float, 3, false, false&gt;(c10::BFloat16*, c10::BFloat16 const*, int, int, int, bool const*, int, bool)</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" t="n">
+        <v>92.672</v>
+      </c>
+      <c r="F17" t="n">
+        <v>12</v>
+      </c>
+      <c r="G17" t="n">
+        <v>7.722666666666666</v>
+      </c>
+      <c r="H17" t="n">
+        <v>7.679</v>
+      </c>
+      <c r="I17" t="n">
+        <v>7.841</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.0598441406007965</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.05792274164344144</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>reduce</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>aten::mean</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>void at::native::reduce_kernel&lt;128, 4, at::native::ReduceOp&lt;c10::BFloat16, at::native::MeanOps&lt;c10::BFloat16, float, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt; &gt;(at::native::ReduceOp&lt;c10::BFloat16, at::native::MeanOps&lt;c10::BFloat16, float, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt;)</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>7</v>
+      </c>
+      <c r="E18" t="n">
+        <v>64.99299999999999</v>
+      </c>
+      <c r="F18" t="n">
+        <v>12</v>
+      </c>
+      <c r="G18" t="n">
+        <v>5.416083333333333</v>
+      </c>
+      <c r="H18" t="n">
+        <v>5.248</v>
+      </c>
+      <c r="I18" t="n">
+        <v>5.536</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.04197006895359512</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.04062254777745369</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>elementwise</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>aten::add_</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E19" t="n">
+        <v>64.864</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="n">
+        <v>64.864</v>
+      </c>
+      <c r="H19" t="n">
+        <v>64.864</v>
+      </c>
+      <c r="I19" t="n">
+        <v>64.864</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.04188676553791938</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.04054191896106899</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CONV_fwd</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>aten::cudnn_convolution</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>void cudnn::engines_precompiled::nhwcToNchwKernel&lt;__nv_bfloat16, __nv_bfloat16, float, true, false, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nhwc2nchw_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>43.488</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>43.488</v>
+      </c>
+      <c r="H20" t="n">
+        <v>43.488</v>
+      </c>
+      <c r="I20" t="n">
+        <v>43.488</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.02808293752640968</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.0271812865654133</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>GEMM</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>aten::addmm</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>std::enable_if&lt;!(false), void&gt;::type internal::gemvx::kernel&lt;int, int, __nv_bfloat16, __nv_bfloat16, __nv_bfloat16, float, false, true, true, false, 7, false, cublasGemvParamsEx&lt;int, cublasGemvTensorStridedBatched&lt;__nv_bfloat16 const&gt;, cublasGemvTensorStridedBatched&lt;__nv_bfloat16 const&gt;, cublasGemvTensorStridedBatched&lt;__nv_bfloat16&gt;, float&gt; &gt;(cublasGemvParamsEx&lt;int, cublasGemvTensorStridedBatched&lt;__nv_bfloat16 const&gt;, cublasGemvTensorStridedBatched&lt;__nv_bfloat16 const&gt;, cublasGemvTensorStridedBatched&lt;__nv_bfloat16&gt;, float&gt;)</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>7</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5.056</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>5.056</v>
+      </c>
+      <c r="H21" t="n">
+        <v>5.056</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5.056</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.003264977284159478</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.003160149578613172</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>aten::upsample_nearest1d</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>void at::native::(anonymous namespace)::upsample_nearest1d_out_frame&lt;c10::BFloat16, &amp;at::native::nearest_neighbor_compute_source_index&gt;(c10::BFloat16 const*, unsigned long, unsigned long, unsigned long, unsigned long, c10::BFloat16*, float)</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>7</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2.305</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2.305</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2.305</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2.305</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.001488483512655775</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.00144069319199038</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>bin_start</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>bin_end</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2.305</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2.36036</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2.36036</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2.41572</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2.41572</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2.47108</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2.47108</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2.52644</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2.52644</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2.5818</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2.5818</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2.63716</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2.63716</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2.69252</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2.69252</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2.74788</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2.74788</v>
+      </c>
+      <c r="B10" t="n">
+        <v>2.80324</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2.80324</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2.8586</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2.8586</v>
+      </c>
+      <c r="B12" t="n">
+        <v>2.91396</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2.91396</v>
+      </c>
+      <c r="B13" t="n">
+        <v>2.96932</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2.96932</v>
+      </c>
+      <c r="B14" t="n">
+        <v>3.02468</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>3.02468</v>
+      </c>
+      <c r="B15" t="n">
+        <v>3.08004</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>3.08004</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3.1354</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>3.1354</v>
+      </c>
+      <c r="B17" t="n">
+        <v>3.19076</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>3.19076</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3.24612</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>3.24612</v>
+      </c>
+      <c r="B19" t="n">
+        <v>3.30148</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>3.30148</v>
+      </c>
+      <c r="B20" t="n">
+        <v>3.35684</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>3.35684</v>
+      </c>
+      <c r="B21" t="n">
+        <v>3.4122</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>3.4122</v>
+      </c>
+      <c r="B22" t="n">
+        <v>3.46756</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>3.46756</v>
+      </c>
+      <c r="B23" t="n">
+        <v>3.52292</v>
+      </c>
+      <c r="C23" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>3.52292</v>
+      </c>
+      <c r="B24" t="n">
+        <v>3.57828</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>3.57828</v>
+      </c>
+      <c r="B25" t="n">
+        <v>3.63364</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>3.63364</v>
+      </c>
+      <c r="B26" t="n">
+        <v>3.689</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>3.689</v>
+      </c>
+      <c r="B27" t="n">
+        <v>3.74436</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>3.74436</v>
+      </c>
+      <c r="B28" t="n">
+        <v>3.79972</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>3.79972</v>
+      </c>
+      <c r="B29" t="n">
+        <v>3.85508</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>3.85508</v>
+      </c>
+      <c r="B30" t="n">
+        <v>3.91044</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>3.91044</v>
+      </c>
+      <c r="B31" t="n">
+        <v>3.9658</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>3.9658</v>
+      </c>
+      <c r="B32" t="n">
+        <v>4.02116</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>4.02116</v>
+      </c>
+      <c r="B33" t="n">
+        <v>4.07652</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>4.07652</v>
+      </c>
+      <c r="B34" t="n">
+        <v>4.13188</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>4.13188</v>
+      </c>
+      <c r="B35" t="n">
+        <v>4.18724</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>4.18724</v>
+      </c>
+      <c r="B36" t="n">
+        <v>4.242599999999999</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>4.242599999999999</v>
+      </c>
+      <c r="B37" t="n">
+        <v>4.29796</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>4.29796</v>
+      </c>
+      <c r="B38" t="n">
+        <v>4.35332</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>4.35332</v>
+      </c>
+      <c r="B39" t="n">
+        <v>4.40868</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>4.40868</v>
+      </c>
+      <c r="B40" t="n">
+        <v>4.46404</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>4.46404</v>
+      </c>
+      <c r="B41" t="n">
+        <v>4.519399999999999</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>4.519399999999999</v>
+      </c>
+      <c r="B42" t="n">
+        <v>4.574759999999999</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>4.574759999999999</v>
+      </c>
+      <c r="B43" t="n">
+        <v>4.63012</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>4.63012</v>
+      </c>
+      <c r="B44" t="n">
+        <v>4.68548</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>4.68548</v>
+      </c>
+      <c r="B45" t="n">
+        <v>4.74084</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>4.74084</v>
+      </c>
+      <c r="B46" t="n">
+        <v>4.7962</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>4.7962</v>
+      </c>
+      <c r="B47" t="n">
+        <v>4.851559999999999</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>4.851559999999999</v>
+      </c>
+      <c r="B48" t="n">
+        <v>4.90692</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>4.90692</v>
+      </c>
+      <c r="B49" t="n">
+        <v>4.96228</v>
+      </c>
+      <c r="C49" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>4.96228</v>
+      </c>
+      <c r="B50" t="n">
+        <v>5.01764</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>5.01764</v>
+      </c>
+      <c r="B51" t="n">
+        <v>5.073</v>
+      </c>
+      <c r="C51" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>5.073</v>
+      </c>
+      <c r="B52" t="n">
+        <v>5.12836</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>5.12836</v>
+      </c>
+      <c r="B53" t="n">
+        <v>5.183719999999999</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>5.183719999999999</v>
+      </c>
+      <c r="B54" t="n">
+        <v>5.23908</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>5.23908</v>
+      </c>
+      <c r="B55" t="n">
+        <v>5.29444</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>5.29444</v>
+      </c>
+      <c r="B56" t="n">
+        <v>5.3498</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>5.3498</v>
+      </c>
+      <c r="B57" t="n">
+        <v>5.40516</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>5.40516</v>
+      </c>
+      <c r="B58" t="n">
+        <v>5.46052</v>
+      </c>
+      <c r="C58" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>5.46052</v>
+      </c>
+      <c r="B59" t="n">
+        <v>5.515879999999999</v>
+      </c>
+      <c r="C59" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>5.515879999999999</v>
+      </c>
+      <c r="B60" t="n">
+        <v>5.57124</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>5.57124</v>
+      </c>
+      <c r="B61" t="n">
+        <v>5.6266</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>5.6266</v>
+      </c>
+      <c r="B62" t="n">
+        <v>5.68196</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>5.68196</v>
+      </c>
+      <c r="B63" t="n">
+        <v>5.73732</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>5.73732</v>
+      </c>
+      <c r="B64" t="n">
+        <v>5.79268</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>5.79268</v>
+      </c>
+      <c r="B65" t="n">
+        <v>5.848039999999999</v>
+      </c>
+      <c r="C65" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>5.848039999999999</v>
+      </c>
+      <c r="B66" t="n">
+        <v>5.9034</v>
+      </c>
+      <c r="C66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>5.9034</v>
+      </c>
+      <c r="B67" t="n">
+        <v>5.95876</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>5.95876</v>
+      </c>
+      <c r="B68" t="n">
+        <v>6.01412</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>6.01412</v>
+      </c>
+      <c r="B69" t="n">
+        <v>6.06948</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>6.06948</v>
+      </c>
+      <c r="B70" t="n">
+        <v>6.12484</v>
+      </c>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>6.12484</v>
+      </c>
+      <c r="B71" t="n">
+        <v>6.180199999999999</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>6.180199999999999</v>
+      </c>
+      <c r="B72" t="n">
+        <v>6.23556</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>6.23556</v>
+      </c>
+      <c r="B73" t="n">
+        <v>6.29092</v>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>6.29092</v>
+      </c>
+      <c r="B74" t="n">
+        <v>6.34628</v>
+      </c>
+      <c r="C74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>6.34628</v>
+      </c>
+      <c r="B75" t="n">
+        <v>6.40164</v>
+      </c>
+      <c r="C75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>6.40164</v>
+      </c>
+      <c r="B76" t="n">
+        <v>6.456999999999999</v>
+      </c>
+      <c r="C76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>6.456999999999999</v>
+      </c>
+      <c r="B77" t="n">
+        <v>6.512359999999999</v>
+      </c>
+      <c r="C77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>6.512359999999999</v>
+      </c>
+      <c r="B78" t="n">
+        <v>6.56772</v>
+      </c>
+      <c r="C78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>6.56772</v>
+      </c>
+      <c r="B79" t="n">
+        <v>6.62308</v>
+      </c>
+      <c r="C79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>6.62308</v>
+      </c>
+      <c r="B80" t="n">
+        <v>6.67844</v>
+      </c>
+      <c r="C80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>6.67844</v>
+      </c>
+      <c r="B81" t="n">
+        <v>6.733799999999999</v>
+      </c>
+      <c r="C81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>6.733799999999999</v>
+      </c>
+      <c r="B82" t="n">
+        <v>6.789159999999999</v>
+      </c>
+      <c r="C82" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>6.789159999999999</v>
+      </c>
+      <c r="B83" t="n">
+        <v>6.844519999999999</v>
+      </c>
+      <c r="C83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>6.844519999999999</v>
+      </c>
+      <c r="B84" t="n">
+        <v>6.89988</v>
+      </c>
+      <c r="C84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>6.89988</v>
+      </c>
+      <c r="B85" t="n">
+        <v>6.95524</v>
+      </c>
+      <c r="C85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>6.95524</v>
+      </c>
+      <c r="B86" t="n">
+        <v>7.0106</v>
+      </c>
+      <c r="C86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>7.0106</v>
+      </c>
+      <c r="B87" t="n">
+        <v>7.065959999999999</v>
+      </c>
+      <c r="C87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>7.065959999999999</v>
+      </c>
+      <c r="B88" t="n">
+        <v>7.121319999999999</v>
+      </c>
+      <c r="C88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>7.121319999999999</v>
+      </c>
+      <c r="B89" t="n">
+        <v>7.176679999999999</v>
+      </c>
+      <c r="C89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>7.176679999999999</v>
+      </c>
+      <c r="B90" t="n">
+        <v>7.23204</v>
+      </c>
+      <c r="C90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>7.23204</v>
+      </c>
+      <c r="B91" t="n">
+        <v>7.2874</v>
+      </c>
+      <c r="C91" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>7.2874</v>
+      </c>
+      <c r="B92" t="n">
+        <v>7.34276</v>
+      </c>
+      <c r="C92" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>7.34276</v>
+      </c>
+      <c r="B93" t="n">
+        <v>7.398119999999999</v>
+      </c>
+      <c r="C93" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>7.398119999999999</v>
+      </c>
+      <c r="B94" t="n">
+        <v>7.453479999999999</v>
+      </c>
+      <c r="C94" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>7.453479999999999</v>
+      </c>
+      <c r="B95" t="n">
+        <v>7.508839999999999</v>
+      </c>
+      <c r="C95" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>7.508839999999999</v>
+      </c>
+      <c r="B96" t="n">
+        <v>7.5642</v>
+      </c>
+      <c r="C96" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>7.5642</v>
+      </c>
+      <c r="B97" t="n">
+        <v>7.61956</v>
+      </c>
+      <c r="C97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>7.61956</v>
+      </c>
+      <c r="B98" t="n">
+        <v>7.67492</v>
+      </c>
+      <c r="C98" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>7.67492</v>
+      </c>
+      <c r="B99" t="n">
+        <v>7.730279999999999</v>
+      </c>
+      <c r="C99" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>7.730279999999999</v>
+      </c>
+      <c r="B100" t="n">
+        <v>7.785639999999999</v>
+      </c>
+      <c r="C100" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>7.785639999999999</v>
+      </c>
+      <c r="B101" t="n">
+        <v>7.841</v>
+      </c>
+      <c r="C101" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parent cpu_op</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Input dims</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Input strides</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Concrete Inputs</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Kernel name</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Short Kernel duration (µs) sum</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Short Kernel count</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Short Kernel duration (µs) mean</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Short Kernel duration (µs) percent of total time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>aten::_softmax</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>((3136, 12, 8, 8), (), ())</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>((768, 64, 8, 1), (), ())</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>('', '-1', 'False')</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>void (anonymous namespace)::softmax_warp_forward&lt;c10::BFloat16, c10::BFloat16, float, 3, false, false&gt;(c10::BFloat16*, c10::BFloat16 const*, int, int, int, bool const*, int, bool)</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>92.672</v>
+      </c>
+      <c r="G2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H2" t="n">
+        <v>7.722666666666666</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.05792274164344144</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>aten::mean</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>((1, 8, 768), (), (), ())</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>((19273728, 2409216, 1), (), (), ())</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>('', '[1]', 'True', '')</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>void at::native::reduce_kernel&lt;128, 4, at::native::ReduceOp&lt;c10::BFloat16, at::native::MeanOps&lt;c10::BFloat16, float, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt; &gt;(at::native::ReduceOp&lt;c10::BFloat16, at::native::MeanOps&lt;c10::BFloat16, float, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt;)</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>64.99299999999999</v>
+      </c>
+      <c r="G3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5.416083333333333</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.04062254777745369</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>aten::mul</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>((3136, 12, 8, 8), ())</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>((768, 64, 8, 1), ())</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>('', '')</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::native::AUnaryFunctor&lt;c10::BFloat16, c10::BFloat16, c10::BFloat16, at::native::binary_internal::MulFunctor&lt;float&gt; &gt;, std::array&lt;char*, 2ul&gt; &gt;(int, at::native::AUnaryFunctor&lt;c10::BFloat16, c10::BFloat16, c10::BFloat16, at::native::binary_internal::MulFunctor&lt;float&gt; &gt;, std::array&lt;char*, 2ul&gt;)</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>60.544</v>
+      </c>
+      <c r="G4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H4" t="n">
+        <v>5.045333333333333</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.03784179115655773</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>aten::copy_</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>((1, 8, 1, 1, 1, 768), (1, 8, 1, 1, 1, 768), ())</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>((6144, 768, 768, 6144, 768, 1), (0, 0, 19268352, 19268352, 768, 1), ())</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>('', '', 'False')</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1}&gt;(at::TensorIteratorBase&amp;, at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1} const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1}&gt;(at::TensorIteratorBase&amp;, at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1} const&amp;)::{lambda(int)#1})</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>41.664</v>
+      </c>
+      <c r="G5" t="n">
+        <v>12</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3.472</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.02604123260350855</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>aten::addmm</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>((400,), (1, 768), (768, 400), (), ())</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>((1,), (19268352, 1), (1, 768), (), ())</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>('', '', '', '1', '1')</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>std::enable_if&lt;!(false), void&gt;::type internal::gemvx::kernel&lt;int, int, __nv_bfloat16, __nv_bfloat16, __nv_bfloat16, float, false, true, true, false, 7, false, cublasGemvParamsEx&lt;int, cublasGemvTensorStridedBatched&lt;__nv_bfloat16 const&gt;, cublasGemvTensorStridedBatched&lt;__nv_bfloat16 const&gt;, cublasGemvTensorStridedBatched&lt;__nv_bfloat16&gt;, float&gt; &gt;(cublasGemvParamsEx&lt;int, cublasGemvTensorStridedBatched&lt;__nv_bfloat16 const&gt;, cublasGemvTensorStridedBatched&lt;__nv_bfloat16 const&gt;, cublasGemvTensorStridedBatched&lt;__nv_bfloat16&gt;, float&gt;)</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>5.056</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5.056</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.003160149578613172</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>aten::copy_</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>((1, 768, 8), (1, 768, 8), ())</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>((6144, 8, 1), (6144, 1, 768), ())</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>('', '', 'False')</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1}&gt;(at::TensorIteratorBase&amp;, at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1} const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1}&gt;(at::TensorIteratorBase&amp;, at::native::direct_copy_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#3}::operator()() const::{lambda()#12}::operator()() const::{lambda(c10::BFloat16)#1} const&amp;)::{lambda(int)#1})</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>3.999</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3.999</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.002499493307926043</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>aten::upsample_nearest1d</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>((1, 768, 8), (), ())</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>((6144, 1, 768), (), ())</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>('', '[128]', '')</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>void at::native::(anonymous namespace)::upsample_nearest1d_out_frame&lt;c10::BFloat16, &amp;at::native::nearest_neighbor_compute_source_index&gt;(c10::BFloat16 const*, unsigned long, unsigned long, unsigned long, unsigned long, c10::BFloat16*, float)</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>2.305</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2.305</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.00144069319199038</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -12428,14 +15165,32 @@
       <c r="N36" t="n">
         <v>3.712242631625875</v>
       </c>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr"/>
+      <c r="O36" t="n">
+        <v>6.144e-06</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0.01172065734863281</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0.4999186330349878</v>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>vector_bf16</t>
+        </is>
+      </c>
+      <c r="S36" t="n">
+        <v>0.00226974951117672</v>
+      </c>
+      <c r="T36" t="n">
+        <v>3.751008785294355e-05</v>
+      </c>
+      <c r="U36" t="n">
+        <v>0.001134690072959298</v>
+      </c>
+      <c r="V36" t="n">
+        <v>1.875199184446587e-05</v>
+      </c>
       <c r="W36" t="n">
         <v>5.416035970052083</v>
       </c>
@@ -12454,12 +15209,24 @@
       <c r="AB36" t="n">
         <v>34.46</v>
       </c>
-      <c r="AC36" t="inlineStr"/>
-      <c r="AD36" t="inlineStr"/>
-      <c r="AE36" t="inlineStr"/>
-      <c r="AF36" t="inlineStr"/>
-      <c r="AG36" t="inlineStr"/>
-      <c r="AH36" t="inlineStr"/>
+      <c r="AC36" t="n">
+        <v>0.002259215510277354</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>0.002220059095920617</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>0.002341823595087458</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>0.001129423929629297</v>
+      </c>
+      <c r="AG36" t="n">
+        <v>0.001109848908489526</v>
+      </c>
+      <c r="AH36" t="n">
+        <v>0.001170721250465203</v>
+      </c>
       <c r="AI36" t="n">
         <v>5.43994140625</v>
       </c>
@@ -12479,9 +15246,13 @@
           <t>[{'name': 'void at::native::reduce_kernel&lt;128, 4, at::native::ReduceOp&lt;c10:...', 'stream': 7, 'mean_duration_us': np.float64(5.42)}]</t>
         </is>
       </c>
-      <c r="AN36" t="inlineStr"/>
+      <c r="AN36" t="inlineStr">
+        <is>
+          <t>{'num_input_elems': 6144, 'num_output_elems': 1, 'dtype_in_out': ('c10::BFloat16', None), 'reduce_type': 'mean'}</t>
+        </is>
+      </c>
       <c r="AO36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP36" t="n">
         <v>0.04102198445609978</v>

</xml_diff>

<commit_message>
fix: deterministic short_kernels_summary sort order
Add string-typed groupby columns as tie-breakers so rows with the same
duration sum have reproducible ordering. Regenerate all reference xlsx.
</commit_message>
<xml_diff>
--- a/tests/traces/h100/facebook_timesformer-base-finetuned-k400__1016002_perf_report.xlsx
+++ b/tests/traces/h100/facebook_timesformer-base-finetuned-k400__1016002_perf_report.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="gpu_timeline" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ops_summary_by_category" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ops_summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ops_unique_args" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="unified_perf_summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="GEMM" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="CONV_fwd" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="BinaryElementwise" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="UnaryElementwise" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Normalization" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Reduce_fwd" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="kernel_summary" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="short_kernel_histogram" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="short_kernels_summary" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gpu_timeline" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ops_summary_by_category" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ops_summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ops_unique_args" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="unified_perf_summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GEMM" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONV_fwd" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BinaryElementwise" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UnaryElementwise" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalization" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduce_fwd" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kernel_summary" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="short_kernel_histogram" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="short_kernels_summary" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4809,7 +4809,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>{'elementwise', 'other'}</t>
+          <t>{'other', 'elementwise'}</t>
         </is>
       </c>
       <c r="H5" t="n">

</xml_diff>